<commit_message>
remove spaces from brand names, add palm oil and soy identification logic
</commit_message>
<xml_diff>
--- a/inputs/all_formula_ingredients_manual_entry.xlsx
+++ b/inputs/all_formula_ingredients_manual_entry.xlsx
@@ -561,7 +561,7 @@
     <t xml:space="preserve">https://us.kendamil.com/products/goat-first-infant-milk</t>
   </si>
   <si>
-    <t xml:space="preserve">Contains Milk.</t>
+    <t xml:space="preserve">whole goat milk, reduced minerals goat whey^, blend of oils (sunflower oil, coconut oil, low erucic acid rapeseed oil), lactose^, galacto-oligosaccharides (gos)^*, less than 2% of: calcium citrate, choline bitartrate, potassium chloride, sodium citrate, magnesium chloride, ascorbic acid, schizochytrium sp. oil^, l-tyrosine, l-phenylalanine, l-tryptophan, potassium hydroxide, inositol, mortierella alpina oil^, l-isoleucine, taurine, calcium phosphate, iron pyrophosphate, nucleotides (cytidine-5'-monophosphate, disodium uridine-5'-monophosphate, adenosine-5'-monophosphate, disodium inosine-5'-monophosphate, disodium guanosine-5'-monophosphate), zinc sulfate, vitamin e acetate, niacinamide, calcium pantothenate, copper sulfate, thiamin hydrochloride, riboflavin, vitamin a acetate, vitamin b6 hydrochloride, manganese sulfate, folic acid^, potassium iodide, sodium selenite, vitamin k1, vitamin d3, biotin, vitamin b12, mixed tocopherols.</t>
   </si>
   <si>
     <t xml:space="preserve">https://us.kendamil.com/products/organic-first-infant-milk</t>
@@ -1066,11 +1066,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1456,7 +1456,7 @@
       <c r="D5" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H5" s="1" t="s">
@@ -1509,7 +1509,7 @@
       <c r="D6" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="2" t="s">
         <v>39</v>
       </c>
       <c r="H6" s="1" t="s">
@@ -1562,7 +1562,7 @@
       <c r="D7" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="2" t="s">
         <v>42</v>
       </c>
       <c r="H7" s="1" t="s">
@@ -1615,7 +1615,7 @@
       <c r="D8" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="2" t="s">
         <v>45</v>
       </c>
       <c r="H8" s="1" t="n">
@@ -1655,7 +1655,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="114.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="114.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="n">
         <v>108</v>
       </c>
@@ -1774,7 +1774,7 @@
       <c r="D11" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="2" t="s">
         <v>56</v>
       </c>
       <c r="H11" s="1" t="s">
@@ -1827,7 +1827,7 @@
       <c r="D12" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="3" t="s">
         <v>60</v>
       </c>
       <c r="H12" s="1" t="n">
@@ -1867,7 +1867,7 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="126.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="126.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="n">
         <v>112</v>
       </c>
@@ -1880,7 +1880,7 @@
       <c r="D13" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="3" t="s">
         <v>63</v>
       </c>
       <c r="H13" s="1" t="n">
@@ -1933,7 +1933,7 @@
       <c r="D14" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="3" t="s">
         <v>66</v>
       </c>
       <c r="H14" s="1" t="n">
@@ -1986,7 +1986,7 @@
       <c r="D15" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="2" t="s">
         <v>70</v>
       </c>
       <c r="H15" s="1" t="s">
@@ -2039,7 +2039,7 @@
       <c r="D16" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="2" t="s">
         <v>73</v>
       </c>
       <c r="H16" s="1" t="n">
@@ -2092,7 +2092,7 @@
       <c r="D17" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E17" s="2" t="s">
         <v>77</v>
       </c>
       <c r="H17" s="1" t="n">
@@ -2145,7 +2145,7 @@
       <c r="D18" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E18" s="2" t="s">
         <v>81</v>
       </c>
       <c r="H18" s="1" t="n">
@@ -2198,7 +2198,7 @@
       <c r="D19" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="E19" s="2" t="s">
         <v>84</v>
       </c>
       <c r="H19" s="1" t="n">
@@ -2251,7 +2251,7 @@
       <c r="D20" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E20" s="2" t="s">
         <v>87</v>
       </c>
       <c r="H20" s="1" t="n">
@@ -2304,7 +2304,7 @@
       <c r="D21" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="E21" s="2" t="s">
         <v>90</v>
       </c>
       <c r="H21" s="1" t="s">
@@ -2357,7 +2357,7 @@
       <c r="D22" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="E22" s="2" t="s">
         <v>93</v>
       </c>
       <c r="H22" s="1" t="n">
@@ -2410,7 +2410,7 @@
       <c r="D23" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="3" t="s">
         <v>96</v>
       </c>
       <c r="H23" s="1" t="s">
@@ -2463,7 +2463,7 @@
       <c r="D24" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="E24" s="2" t="s">
         <v>99</v>
       </c>
       <c r="H24" s="1" t="s">
@@ -2516,7 +2516,7 @@
       <c r="D25" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E25" s="3" t="s">
         <v>102</v>
       </c>
       <c r="H25" s="1" t="n">
@@ -2569,7 +2569,7 @@
       <c r="D26" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="E26" s="2" t="s">
         <v>105</v>
       </c>
       <c r="H26" s="1" t="n">
@@ -2622,7 +2622,7 @@
       <c r="D27" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="E27" s="2" t="s">
         <v>108</v>
       </c>
       <c r="H27" s="1" t="n">
@@ -2675,7 +2675,7 @@
       <c r="D28" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="E28" s="2" t="s">
         <v>111</v>
       </c>
       <c r="H28" s="1" t="n">
@@ -2728,7 +2728,7 @@
       <c r="D29" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="E29" s="3" t="s">
+      <c r="E29" s="2" t="s">
         <v>114</v>
       </c>
       <c r="H29" s="1" t="s">
@@ -2781,7 +2781,7 @@
       <c r="D30" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="E30" s="3" t="s">
+      <c r="E30" s="2" t="s">
         <v>117</v>
       </c>
       <c r="H30" s="1" t="n">
@@ -2834,7 +2834,7 @@
       <c r="D31" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="E31" s="3" t="s">
+      <c r="E31" s="2" t="s">
         <v>120</v>
       </c>
       <c r="H31" s="1" t="n">
@@ -2887,7 +2887,7 @@
       <c r="D32" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="E32" s="2" t="s">
         <v>117</v>
       </c>
       <c r="H32" s="1" t="n">
@@ -2940,7 +2940,7 @@
       <c r="D33" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="E33" s="3" t="s">
+      <c r="E33" s="2" t="s">
         <v>125</v>
       </c>
       <c r="H33" s="1" t="s">
@@ -2993,7 +2993,7 @@
       <c r="D34" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="E34" s="3" t="s">
+      <c r="E34" s="2" t="s">
         <v>128</v>
       </c>
       <c r="H34" s="1" t="n">
@@ -3046,7 +3046,7 @@
       <c r="D35" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="E35" s="3" t="s">
+      <c r="E35" s="2" t="s">
         <v>131</v>
       </c>
       <c r="H35" s="1" t="n">
@@ -3099,7 +3099,7 @@
       <c r="D36" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="E36" s="3" t="s">
+      <c r="E36" s="2" t="s">
         <v>131</v>
       </c>
       <c r="H36" s="1" t="n">
@@ -3152,7 +3152,7 @@
       <c r="D37" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="E37" s="3" t="s">
+      <c r="E37" s="2" t="s">
         <v>135</v>
       </c>
       <c r="H37" s="1" t="n">
@@ -3205,7 +3205,7 @@
       <c r="D38" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="E38" s="3" t="s">
+      <c r="E38" s="2" t="s">
         <v>138</v>
       </c>
       <c r="H38" s="1" t="n">
@@ -3258,7 +3258,7 @@
       <c r="D39" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="E39" s="3" t="s">
+      <c r="E39" s="2" t="s">
         <v>142</v>
       </c>
       <c r="H39" s="1" t="n">
@@ -3311,7 +3311,7 @@
       <c r="D40" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="E40" s="3" t="s">
+      <c r="E40" s="2" t="s">
         <v>144</v>
       </c>
       <c r="H40" s="1" t="s">
@@ -3364,7 +3364,7 @@
       <c r="D41" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="E41" s="3" t="s">
+      <c r="E41" s="2" t="s">
         <v>148</v>
       </c>
       <c r="H41" s="1" t="s">
@@ -3417,7 +3417,7 @@
       <c r="D42" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="E42" s="3" t="s">
+      <c r="E42" s="2" t="s">
         <v>150</v>
       </c>
       <c r="H42" s="1" t="n">
@@ -3470,7 +3470,7 @@
       <c r="D43" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="E43" s="3" t="s">
+      <c r="E43" s="2" t="s">
         <v>153</v>
       </c>
       <c r="H43" s="1" t="s">
@@ -3523,7 +3523,7 @@
       <c r="D44" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="E44" s="3" t="s">
+      <c r="E44" s="2" t="s">
         <v>157</v>
       </c>
       <c r="H44" s="1" t="s">
@@ -3576,7 +3576,7 @@
       <c r="D45" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="E45" s="3" t="s">
+      <c r="E45" s="2" t="s">
         <v>160</v>
       </c>
       <c r="H45" s="1" t="n">
@@ -3775,7 +3775,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="114.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="n">
         <v>148</v>
       </c>
@@ -3788,7 +3788,7 @@
       <c r="D49" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="E49" s="2" t="s">
+      <c r="E49" s="4" t="s">
         <v>175</v>
       </c>
       <c r="H49" s="1" t="n">

</xml_diff>